<commit_message>
Fix frontend runtime bug, improve backend CORS/cache, add tests and conversiones UI
</commit_message>
<xml_diff>
--- a/data/barra su nombre original es (inventario valorizado costos) sin el parentesis.xlsx
+++ b/data/barra su nombre original es (inventario valorizado costos) sin el parentesis.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24527"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\licores\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AFE607F5-EE1E-4874-BFC1-0EB953DC7FFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04A78A2D-64F9-4EA9-A181-6A81B0B0A8D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13140"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="barra su nombre original es (in" sheetId="1" r:id="rId1"/>
@@ -1174,8 +1174,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="16" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color indexed="8"/>
@@ -1263,6 +1263,10 @@
       <color indexed="8"/>
       <name val="MS Sans Serif"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="MS Sans Serif"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1284,7 +1288,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -1317,6 +1321,7 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1630,11 +1635,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A2:L189"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1645,7 +1650,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>3</v>
       </c>
@@ -1653,7 +1658,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
         <v>5</v>
       </c>
@@ -1664,12 +1669,12 @@
         <v>381</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="F5" s="6" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" s="15" t="s">
         <v>380</v>
       </c>
@@ -1686,7 +1691,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" s="8" t="s">
         <v>11</v>
       </c>
@@ -1712,7 +1717,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" s="9" t="s">
         <v>18</v>
       </c>
@@ -1738,7 +1743,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9" s="9" t="s">
         <v>21</v>
       </c>
@@ -1764,7 +1769,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A10" s="9" t="s">
         <v>23</v>
       </c>
@@ -1790,7 +1795,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A11" s="9" t="s">
         <v>25</v>
       </c>
@@ -1816,7 +1821,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12" s="9" t="s">
         <v>27</v>
       </c>
@@ -1842,7 +1847,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A13" s="9" t="s">
         <v>29</v>
       </c>
@@ -1868,7 +1873,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14" s="9" t="s">
         <v>31</v>
       </c>
@@ -1894,7 +1899,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A15" s="9" t="s">
         <v>33</v>
       </c>
@@ -1920,7 +1925,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16" s="9" t="s">
         <v>35</v>
       </c>
@@ -1946,7 +1951,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17" s="9" t="s">
         <v>37</v>
       </c>
@@ -1972,7 +1977,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A18" s="9" t="s">
         <v>39</v>
       </c>
@@ -1998,7 +2003,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19" s="9" t="s">
         <v>41</v>
       </c>
@@ -2024,7 +2029,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A20" s="9" t="s">
         <v>43</v>
       </c>
@@ -2050,7 +2055,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A21" s="9" t="s">
         <v>45</v>
       </c>
@@ -2076,7 +2081,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A22" s="9" t="s">
         <v>47</v>
       </c>
@@ -2102,7 +2107,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A23" s="9" t="s">
         <v>49</v>
       </c>
@@ -2128,7 +2133,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A24" s="9" t="s">
         <v>51</v>
       </c>
@@ -2154,7 +2159,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A25" s="9" t="s">
         <v>53</v>
       </c>
@@ -2180,7 +2185,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A26" s="9" t="s">
         <v>55</v>
       </c>
@@ -2206,7 +2211,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A27" s="9" t="s">
         <v>57</v>
       </c>
@@ -2232,7 +2237,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A28" s="9" t="s">
         <v>59</v>
       </c>
@@ -2258,7 +2263,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A29" s="9" t="s">
         <v>61</v>
       </c>
@@ -2284,7 +2289,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A30" s="9" t="s">
         <v>63</v>
       </c>
@@ -2310,7 +2315,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A31" s="9" t="s">
         <v>65</v>
       </c>
@@ -2336,7 +2341,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A32" s="9" t="s">
         <v>67</v>
       </c>
@@ -2362,7 +2367,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A33" s="9" t="s">
         <v>69</v>
       </c>
@@ -2388,7 +2393,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A34" s="9" t="s">
         <v>71</v>
       </c>
@@ -2414,7 +2419,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A35" s="9" t="s">
         <v>73</v>
       </c>
@@ -2440,7 +2445,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A36" s="9" t="s">
         <v>75</v>
       </c>
@@ -2466,7 +2471,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A37" s="9" t="s">
         <v>77</v>
       </c>
@@ -2492,7 +2497,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A38" s="9" t="s">
         <v>79</v>
       </c>
@@ -2518,7 +2523,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A39" s="9" t="s">
         <v>81</v>
       </c>
@@ -2544,7 +2549,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A40" s="9" t="s">
         <v>83</v>
       </c>
@@ -2570,7 +2575,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A41" s="9" t="s">
         <v>85</v>
       </c>
@@ -2596,7 +2601,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A42" s="9" t="s">
         <v>87</v>
       </c>
@@ -2622,7 +2627,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A43" s="9" t="s">
         <v>89</v>
       </c>
@@ -2648,7 +2653,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A44" s="9" t="s">
         <v>91</v>
       </c>
@@ -2674,7 +2679,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A45" s="9" t="s">
         <v>93</v>
       </c>
@@ -2700,7 +2705,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A46" s="9" t="s">
         <v>95</v>
       </c>
@@ -2726,7 +2731,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A47" s="9" t="s">
         <v>97</v>
       </c>
@@ -2752,7 +2757,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A48" s="9" t="s">
         <v>99</v>
       </c>
@@ -2778,7 +2783,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A49" s="9" t="s">
         <v>101</v>
       </c>
@@ -2804,7 +2809,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A50" s="9" t="s">
         <v>103</v>
       </c>
@@ -2830,7 +2835,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A51" s="9" t="s">
         <v>105</v>
       </c>
@@ -2856,7 +2861,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A52" s="9" t="s">
         <v>107</v>
       </c>
@@ -2882,7 +2887,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A53" s="9" t="s">
         <v>109</v>
       </c>
@@ -2908,7 +2913,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A54" s="9" t="s">
         <v>111</v>
       </c>
@@ -2934,7 +2939,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A55" s="9" t="s">
         <v>113</v>
       </c>
@@ -2960,7 +2965,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A56" s="9" t="s">
         <v>115</v>
       </c>
@@ -2986,7 +2991,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A57" s="9" t="s">
         <v>117</v>
       </c>
@@ -3012,7 +3017,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A58" s="9" t="s">
         <v>119</v>
       </c>
@@ -3038,7 +3043,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A59" s="9" t="s">
         <v>121</v>
       </c>
@@ -3064,7 +3069,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A60" s="9" t="s">
         <v>123</v>
       </c>
@@ -3090,7 +3095,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A61" s="9" t="s">
         <v>125</v>
       </c>
@@ -3116,7 +3121,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A62" s="9" t="s">
         <v>127</v>
       </c>
@@ -3142,7 +3147,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A63" s="9" t="s">
         <v>129</v>
       </c>
@@ -3168,7 +3173,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A64" s="9" t="s">
         <v>131</v>
       </c>
@@ -3194,7 +3199,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A65" s="9" t="s">
         <v>133</v>
       </c>
@@ -3220,7 +3225,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A66" s="9" t="s">
         <v>135</v>
       </c>
@@ -3246,7 +3251,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A67" s="9" t="s">
         <v>137</v>
       </c>
@@ -3272,7 +3277,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A68" s="9" t="s">
         <v>139</v>
       </c>
@@ -3298,7 +3303,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A69" s="9" t="s">
         <v>141</v>
       </c>
@@ -3324,7 +3329,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A70" s="9" t="s">
         <v>143</v>
       </c>
@@ -3350,7 +3355,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A71" s="9" t="s">
         <v>145</v>
       </c>
@@ -3376,7 +3381,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A72" s="9" t="s">
         <v>147</v>
       </c>
@@ -3402,7 +3407,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A73" s="9" t="s">
         <v>149</v>
       </c>
@@ -3428,7 +3433,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A74" s="9" t="s">
         <v>151</v>
       </c>
@@ -3454,7 +3459,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A75" s="9" t="s">
         <v>153</v>
       </c>
@@ -3480,7 +3485,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A76" s="9" t="s">
         <v>155</v>
       </c>
@@ -3506,7 +3511,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A77" s="9" t="s">
         <v>157</v>
       </c>
@@ -3532,7 +3537,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A78" s="9" t="s">
         <v>159</v>
       </c>
@@ -3558,7 +3563,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A79" s="9" t="s">
         <v>161</v>
       </c>
@@ -3584,7 +3589,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A80" s="9" t="s">
         <v>163</v>
       </c>
@@ -3610,7 +3615,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A81" s="9" t="s">
         <v>165</v>
       </c>
@@ -3636,7 +3641,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A82" s="9" t="s">
         <v>167</v>
       </c>
@@ -3662,7 +3667,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A83" s="9" t="s">
         <v>169</v>
       </c>
@@ -3688,7 +3693,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A84" s="9" t="s">
         <v>171</v>
       </c>
@@ -3714,7 +3719,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A85" s="9" t="s">
         <v>173</v>
       </c>
@@ -3740,7 +3745,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A86" s="9" t="s">
         <v>175</v>
       </c>
@@ -3766,7 +3771,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A87" s="9" t="s">
         <v>177</v>
       </c>
@@ -3792,7 +3797,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A88" s="9" t="s">
         <v>179</v>
       </c>
@@ -3818,7 +3823,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A89" s="9" t="s">
         <v>181</v>
       </c>
@@ -3844,7 +3849,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A90" s="9" t="s">
         <v>183</v>
       </c>
@@ -3870,7 +3875,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A91" s="9" t="s">
         <v>185</v>
       </c>
@@ -3896,7 +3901,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A92" s="9" t="s">
         <v>187</v>
       </c>
@@ -3922,7 +3927,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A93" s="9" t="s">
         <v>189</v>
       </c>
@@ -3948,7 +3953,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A94" s="9" t="s">
         <v>191</v>
       </c>
@@ -3974,7 +3979,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A95" s="9" t="s">
         <v>193</v>
       </c>
@@ -4000,7 +4005,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A96" s="9" t="s">
         <v>195</v>
       </c>
@@ -4026,7 +4031,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A97" s="9" t="s">
         <v>197</v>
       </c>
@@ -4052,7 +4057,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A98" s="9" t="s">
         <v>199</v>
       </c>
@@ -4078,7 +4083,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A99" s="9" t="s">
         <v>201</v>
       </c>
@@ -4104,7 +4109,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A100" s="9" t="s">
         <v>203</v>
       </c>
@@ -4130,7 +4135,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A101" s="9" t="s">
         <v>205</v>
       </c>
@@ -4156,7 +4161,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A102" s="9" t="s">
         <v>207</v>
       </c>
@@ -4182,7 +4187,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A103" s="9" t="s">
         <v>209</v>
       </c>
@@ -4208,7 +4213,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A104" s="9" t="s">
         <v>211</v>
       </c>
@@ -4234,7 +4239,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A105" s="9" t="s">
         <v>213</v>
       </c>
@@ -4260,7 +4265,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A106" s="9" t="s">
         <v>215</v>
       </c>
@@ -4286,7 +4291,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A107" s="9" t="s">
         <v>217</v>
       </c>
@@ -4312,7 +4317,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A108" s="9" t="s">
         <v>219</v>
       </c>
@@ -4338,7 +4343,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A109" s="9" t="s">
         <v>221</v>
       </c>
@@ -4364,7 +4369,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A110" s="9" t="s">
         <v>223</v>
       </c>
@@ -4390,7 +4395,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A111" s="9" t="s">
         <v>225</v>
       </c>
@@ -4416,7 +4421,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A112" s="9" t="s">
         <v>227</v>
       </c>
@@ -4442,7 +4447,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A113" s="9" t="s">
         <v>229</v>
       </c>
@@ -4468,7 +4473,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A114" s="9" t="s">
         <v>231</v>
       </c>
@@ -4494,7 +4499,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A115" s="9" t="s">
         <v>233</v>
       </c>
@@ -4520,7 +4525,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A116" s="9" t="s">
         <v>235</v>
       </c>
@@ -4546,7 +4551,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A117" s="9" t="s">
         <v>237</v>
       </c>
@@ -4572,7 +4577,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A118" s="9" t="s">
         <v>239</v>
       </c>
@@ -4598,7 +4603,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A119" s="9" t="s">
         <v>241</v>
       </c>
@@ -4624,7 +4629,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A120" s="9" t="s">
         <v>243</v>
       </c>
@@ -4650,7 +4655,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A121" s="9" t="s">
         <v>245</v>
       </c>
@@ -4676,7 +4681,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A122" s="9" t="s">
         <v>247</v>
       </c>
@@ -4702,7 +4707,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A123" s="9" t="s">
         <v>249</v>
       </c>
@@ -4728,7 +4733,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A124" s="9" t="s">
         <v>251</v>
       </c>
@@ -4754,7 +4759,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A125" s="9" t="s">
         <v>253</v>
       </c>
@@ -4780,7 +4785,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A126" s="9" t="s">
         <v>255</v>
       </c>
@@ -4806,7 +4811,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A127" s="9" t="s">
         <v>257</v>
       </c>
@@ -4832,7 +4837,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A128" s="9" t="s">
         <v>259</v>
       </c>
@@ -4858,7 +4863,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A129" s="9" t="s">
         <v>261</v>
       </c>
@@ -4884,7 +4889,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A130" s="9" t="s">
         <v>263</v>
       </c>
@@ -4910,7 +4915,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A131" s="9" t="s">
         <v>265</v>
       </c>
@@ -4936,7 +4941,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A132" s="9" t="s">
         <v>267</v>
       </c>
@@ -4962,7 +4967,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A133" s="9" t="s">
         <v>269</v>
       </c>
@@ -4988,7 +4993,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A134" s="9" t="s">
         <v>271</v>
       </c>
@@ -5014,7 +5019,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="135" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A135" s="9" t="s">
         <v>273</v>
       </c>
@@ -5040,7 +5045,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A136" s="9" t="s">
         <v>275</v>
       </c>
@@ -5066,7 +5071,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A137" s="9" t="s">
         <v>277</v>
       </c>
@@ -5092,7 +5097,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A138" s="9" t="s">
         <v>279</v>
       </c>
@@ -5118,7 +5123,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A139" s="9" t="s">
         <v>281</v>
       </c>
@@ -5144,7 +5149,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A140" s="9" t="s">
         <v>283</v>
       </c>
@@ -5170,7 +5175,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A141" s="9" t="s">
         <v>285</v>
       </c>
@@ -5196,7 +5201,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A142" s="9" t="s">
         <v>287</v>
       </c>
@@ -5222,7 +5227,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A143" s="9" t="s">
         <v>289</v>
       </c>
@@ -5248,7 +5253,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A144" s="9" t="s">
         <v>291</v>
       </c>
@@ -5274,7 +5279,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="145" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A145" s="9" t="s">
         <v>293</v>
       </c>
@@ -5300,7 +5305,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A146" s="9" t="s">
         <v>295</v>
       </c>
@@ -5326,7 +5331,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A147" s="9" t="s">
         <v>297</v>
       </c>
@@ -5352,7 +5357,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="148" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A148" s="9" t="s">
         <v>299</v>
       </c>
@@ -5378,7 +5383,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="149" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A149" s="9" t="s">
         <v>301</v>
       </c>
@@ -5404,7 +5409,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="150" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A150" s="9" t="s">
         <v>303</v>
       </c>
@@ -5430,7 +5435,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="151" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A151" s="9" t="s">
         <v>305</v>
       </c>
@@ -5456,7 +5461,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="152" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A152" s="9" t="s">
         <v>307</v>
       </c>
@@ -5482,7 +5487,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="153" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A153" s="9" t="s">
         <v>309</v>
       </c>
@@ -5508,7 +5513,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A154" s="9" t="s">
         <v>311</v>
       </c>
@@ -5534,7 +5539,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A155" s="9" t="s">
         <v>313</v>
       </c>
@@ -5560,7 +5565,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A156" s="9" t="s">
         <v>315</v>
       </c>
@@ -5586,7 +5591,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A157" s="9" t="s">
         <v>317</v>
       </c>
@@ -5612,7 +5617,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A158" s="9" t="s">
         <v>319</v>
       </c>
@@ -5638,7 +5643,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="159" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A159" s="9" t="s">
         <v>321</v>
       </c>
@@ -5664,7 +5669,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="160" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A160" s="9" t="s">
         <v>323</v>
       </c>
@@ -5690,7 +5695,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A161" s="9" t="s">
         <v>325</v>
       </c>
@@ -5716,7 +5721,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A162" s="9" t="s">
         <v>327</v>
       </c>
@@ -5742,7 +5747,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="163" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A163" s="9" t="s">
         <v>329</v>
       </c>
@@ -5768,7 +5773,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="164" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A164" s="9" t="s">
         <v>331</v>
       </c>
@@ -5794,7 +5799,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="165" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A165" s="9" t="s">
         <v>333</v>
       </c>
@@ -5820,7 +5825,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="166" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A166" s="9" t="s">
         <v>335</v>
       </c>
@@ -5846,7 +5851,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="167" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A167" s="9" t="s">
         <v>337</v>
       </c>
@@ -5872,7 +5877,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="168" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A168" s="9" t="s">
         <v>339</v>
       </c>
@@ -5898,7 +5903,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A169" s="9" t="s">
         <v>341</v>
       </c>
@@ -5924,7 +5929,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="170" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A170" s="9" t="s">
         <v>343</v>
       </c>
@@ -5950,7 +5955,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A171" s="9" t="s">
         <v>345</v>
       </c>
@@ -5976,7 +5981,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A172" s="9" t="s">
         <v>347</v>
       </c>
@@ -6002,7 +6007,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="173" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A173" s="9" t="s">
         <v>349</v>
       </c>
@@ -6028,7 +6033,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="174" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A174" s="9" t="s">
         <v>351</v>
       </c>
@@ -6054,7 +6059,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A175" s="9" t="s">
         <v>353</v>
       </c>
@@ -6080,8 +6085,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="176" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A176" s="9" t="s">
+    <row r="176" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A176" s="16" t="s">
         <v>355</v>
       </c>
       <c r="D176" s="9" t="s">
@@ -6106,7 +6111,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A177" s="9" t="s">
         <v>357</v>
       </c>
@@ -6132,7 +6137,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A178" s="9" t="s">
         <v>359</v>
       </c>
@@ -6158,7 +6163,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="179" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A179" s="9" t="s">
         <v>361</v>
       </c>
@@ -6184,7 +6189,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A180" s="9" t="s">
         <v>363</v>
       </c>
@@ -6210,7 +6215,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A181" s="9" t="s">
         <v>365</v>
       </c>
@@ -6236,7 +6241,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="182" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A182" s="9" t="s">
         <v>367</v>
       </c>
@@ -6262,7 +6267,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="183" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A183" s="9" t="s">
         <v>369</v>
       </c>
@@ -6288,7 +6293,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="184" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A184" s="9" t="s">
         <v>371</v>
       </c>
@@ -6314,7 +6319,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="185" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A185" s="9" t="s">
         <v>373</v>
       </c>
@@ -6340,7 +6345,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="186" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A186" s="9" t="s">
         <v>375</v>
       </c>
@@ -6366,7 +6371,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="187" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A187" s="12" t="s">
         <v>377</v>
       </c>
@@ -6380,17 +6385,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="188" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A188" s="13" t="s">
         <v>378</v>
       </c>
     </row>
-    <row r="189" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:12" x14ac:dyDescent="0.2">
       <c r="K189" s="14" t="s">
         <v>379</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="16" type="noConversion"/>
   <pageMargins left="0.24788568095654706" right="0.24788568095654706" top="0.24788568095654706" bottom="0.24788568095654706" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="0" r:id="rId1"/>
 </worksheet>

</xml_diff>